<commit_message>
Update Livre Fine Misato-Chuo with full primary DD (Documents 1-3 + Hirose-san inquiry): R8 tax eval, rent roll, Orix/au Jibun 35yr loans, 1/2 road share & joint land use agreement, and sync 5-tab datastore
</commit_message>
<xml_diff>
--- a/data/real_estate_datastore.xlsx
+++ b/data/real_estate_datastore.xlsx
@@ -6319,13 +6319,13 @@
         </is>
       </c>
       <c r="E13" s="0">
-        <v>97.1</v>
+        <v>91.4</v>
       </c>
       <c r="F13" s="0">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G13" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13" s="0">
         <v>0</v>
@@ -40785,59 +40785,59 @@
       </c>
     </row>
     <row r="401">
-      <c r="A401" s="0" t="inlineStr">
+      <c r="A401" s="3" t="inlineStr">
         <is>
           <t>livre-fine-misato-chuo</t>
         </is>
       </c>
-      <c r="B401" s="0" t="inlineStr">
+      <c r="B401" s="3" t="inlineStr">
         <is>
           <t>CHK_15</t>
         </is>
       </c>
-      <c r="C401" s="0" t="inlineStr">
+      <c r="C401" s="3" t="inlineStr">
         <is>
           <t>3.건물/적법</t>
         </is>
       </c>
-      <c r="D401" s="0" t="inlineStr">
+      <c r="D401" s="3" t="inlineStr">
         <is>
           <t>has_inspection_cert</t>
         </is>
       </c>
-      <c r="E401" s="0" t="inlineStr">
+      <c r="E401" s="3" t="inlineStr">
         <is>
           <t>준공검사필증(検査済証) 취득 여부</t>
         </is>
       </c>
-      <c r="F401" s="0" t="inlineStr">
+      <c r="F401" s="3" t="inlineStr">
         <is>
           <t>検査済証の有無</t>
         </is>
       </c>
-      <c r="G401" s="0" t="inlineStr">
+      <c r="G401" s="3" t="inlineStr">
         <is>
           <t>유 (2021.2 신축·오릭스/au지분은행 열화3급 35년 융자평가 확인완료 / 원본사본 징구예정)</t>
         </is>
       </c>
-      <c r="H401" s="0" t="inlineStr">
-        <is>
-          <t>COLLECTED</t>
-        </is>
-      </c>
-      <c r="I401" s="0" t="inlineStr">
-        <is>
-          <t>검사필증/대장</t>
-        </is>
-      </c>
-      <c r="J401" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K401" s="0" t="inlineStr">
-        <is>
-          <t/>
+      <c r="H401" s="3" t="inlineStr">
+        <is>
+          <t>ESTIMATED</t>
+        </is>
+      </c>
+      <c r="I401" s="3" t="inlineStr">
+        <is>
+          <t>오릭스·au지분 35년 융자평가 확인 (원본사본 미징구)</t>
+        </is>
+      </c>
+      <c r="J401" s="3" t="inlineStr">
+        <is>
+          <t>준공검사필증(検査済証) 및 열화대책등급 3급 주택성능평가서 사본, 프로판가스(LPG) 무상대여 약정서 유무 공유 요청</t>
+        </is>
+      </c>
+      <c r="K401" s="3" t="inlineStr">
+        <is>
+          <t>検査済証および劣化対策等級3級の住宅性能評価書の写し、ならびにプロパンガス無償貸与契約の有無のご確認</t>
         </is>
       </c>
     </row>
@@ -41070,59 +41070,59 @@
       </c>
     </row>
     <row r="406">
-      <c r="A406" s="0" t="inlineStr">
+      <c r="A406" s="3" t="inlineStr">
         <is>
           <t>livre-fine-misato-chuo</t>
         </is>
       </c>
-      <c r="B406" s="0" t="inlineStr">
+      <c r="B406" s="3" t="inlineStr">
         <is>
           <t>CHK_20</t>
         </is>
       </c>
-      <c r="C406" s="0" t="inlineStr">
+      <c r="C406" s="3" t="inlineStr">
         <is>
           <t>4.렌트롤</t>
         </is>
       </c>
-      <c r="D406" s="0" t="inlineStr">
+      <c r="D406" s="3" t="inlineStr">
         <is>
           <t>rent_roll_tenant_types</t>
         </is>
       </c>
-      <c r="E406" s="0" t="inlineStr">
+      <c r="E406" s="3" t="inlineStr">
         <is>
           <t>호실별 입주자 속성(법인/직장인/학생/보증회사)</t>
         </is>
       </c>
-      <c r="F406" s="0" t="inlineStr">
+      <c r="F406" s="3" t="inlineStr">
         <is>
           <t>入居者属性・保証会社加入状況</t>
         </is>
       </c>
-      <c r="G406" s="0" t="inlineStr">
+      <c r="G406" s="3" t="inlineStr">
         <is>
           <t>속성 확인 (12실)</t>
         </is>
       </c>
-      <c r="H406" s="0" t="inlineStr">
-        <is>
-          <t>COLLECTED</t>
-        </is>
-      </c>
-      <c r="I406" s="0" t="inlineStr">
-        <is>
-          <t>렌트롤 상세판</t>
-        </is>
-      </c>
-      <c r="J406" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K406" s="0" t="inlineStr">
-        <is>
-          <t/>
+      <c r="H406" s="3" t="inlineStr">
+        <is>
+          <t>ESTIMATED</t>
+        </is>
+      </c>
+      <c r="I406" s="3" t="inlineStr">
+        <is>
+          <t>공식 렌트롤 (敷金·RC 『調査中』 표기)</t>
+        </is>
+      </c>
+      <c r="J406" s="3" t="inlineStr">
+        <is>
+          <t>렌트롤상 『調査中』인 전 호실 시키킨(敷金)·RC 확정 금액 및 서브리스 해지 승계 무보증 6세대의 최근 6개월 수납 내역 확인</t>
+        </is>
+      </c>
+      <c r="K406" s="3" t="inlineStr">
+        <is>
+          <t>レントロール上「調査中」となっている各戸敷金・RCの確定額、および保証会社無しの6戸における直近6ヶ月の家賃入金状況のご確認</t>
         </is>
       </c>
     </row>
@@ -41682,17 +41682,17 @@
       </c>
       <c r="I416" s="3" t="inlineStr">
         <is>
-          <t>표준산식 역산 추정</t>
+          <t>공시지가 기반 노선가 산정 / 본하수 부담금 시청 조사중</t>
         </is>
       </c>
       <c r="J416" s="3" t="inlineStr">
         <is>
-          <t>국세청 최신 노선가 기준 토지 적산단가 대조</t>
+          <t>현재 미사토시청에 조사 중인 하수도 수익자부담금 확정액 및 본하수 접속공사(세금포함 약 180만 엔) 상세 견적서 공유 요청</t>
         </is>
       </c>
       <c r="K416" s="3" t="inlineStr">
         <is>
-          <t>国税庁路線価図に基づく土地評価額の算出</t>
+          <t>現在三郷市役所にて調査中の下水道受益者負担金の確定額、および本下水接続工事（税込約180万円）の詳細見積書のご共有</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Karen Residence Nishitakenotsuka with Okada Real Estate confirmed rent roll & leasing flyers (KO/JA reports, datastore, dual-portal)
</commit_message>
<xml_diff>
--- a/data/real_estate_datastore.xlsx
+++ b/data/real_estate_datastore.xlsx
@@ -7344,7 +7344,7 @@
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
@@ -7353,16 +7353,16 @@
         </is>
       </c>
       <c r="E15" s="0">
-        <v>74.3</v>
+        <v>77.1</v>
       </c>
       <c r="F15" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G15" s="0">
+        <v>3</v>
+      </c>
+      <c r="H15" s="0">
         <v>5</v>
-      </c>
-      <c r="H15" s="0">
-        <v>4</v>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="AQ15" s="0" t="inlineStr">
         <is>
-          <t>1LDK(32.57~33.01㎡)×6호 [1층] + 2LDK 메조네트(70.48~71.76㎡, 1F현관+2·3F)×6호</t>
+          <t>1LDK(32.78~33.01㎡)×5호 + 1DK(32.57㎡)×1호 [1층] + 2LDK 메조네트(70.48~71.76㎡, 임대도면 면적 미기재)×6호 [2~3층]</t>
         </is>
       </c>
       <c r="AR15" s="0" t="inlineStr">
@@ -7552,16 +7552,16 @@
         <v>0</v>
       </c>
       <c r="AZ15" s="0">
-        <v>21672000</v>
+        <v>21768000</v>
       </c>
       <c r="BA15" s="0">
-        <v>23868000</v>
+        <v>21768000</v>
       </c>
       <c r="BB15" s="0">
-        <v>6.57</v>
+        <v>6.6</v>
       </c>
       <c r="BC15" s="0">
-        <v>7.23</v>
+        <v>6.6</v>
       </c>
       <c r="BD15" s="2" t="inlineStr">
         <is>
@@ -7569,16 +7569,16 @@
         </is>
       </c>
       <c r="BE15" s="0">
-        <v>3663600</v>
+        <v>3668400</v>
       </c>
       <c r="BF15" s="0">
-        <v>16.9</v>
+        <v>16.85</v>
       </c>
       <c r="BG15" s="0">
-        <v>16924800</v>
+        <v>17011200</v>
       </c>
       <c r="BH15" s="0">
-        <v>5.13</v>
+        <v>5.15</v>
       </c>
       <c r="BI15" s="0">
         <v>382500</v>
@@ -7617,19 +7617,19 @@
         <v>12028923</v>
       </c>
       <c r="BU15" s="0">
-        <v>4895877</v>
+        <v>4982277</v>
       </c>
       <c r="BV15" s="0">
-        <v>3283663</v>
+        <v>3348463</v>
       </c>
       <c r="BW15" s="0">
         <v>1.41</v>
       </c>
       <c r="BX15" s="0">
-        <v>2.13</v>
+        <v>2.14</v>
       </c>
       <c r="BY15" s="0">
-        <v>72.4</v>
+        <v>72.1</v>
       </c>
       <c r="BZ15" s="0">
         <v>3.3</v>
@@ -7638,7 +7638,7 @@
         <v>91219000</v>
       </c>
       <c r="CB15" s="0">
-        <v>5.37</v>
+        <v>5.46</v>
       </c>
       <c r="CC15" s="0" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
         <v>5.0</v>
       </c>
       <c r="CN15" s="0">
-        <v>-2196000</v>
+        <v>-2100000</v>
       </c>
       <c r="CO15" s="0">
         <v>2.8</v>
@@ -7711,7 +7711,7 @@
       </c>
       <c r="CV15" s="0" t="inlineStr">
         <is>
-          <t>C+ 등급 (61/100점 | 19.6/30점) — 타케노츠카역(고가화 완공·에키아 개업·히비야선 직통) 도보 3분, 근린상업지역 116.35평 토지 + 2026년 신축 목조 3층(열화3급 상당, 605.17㎡, 적산비율 75.8%). 단, ①마이소쿠 임대료 합산 오차(-66만 엔/년) 및 실제 포털(SUUMO) 2LDK 모집가 인하(20만→17.5만~18.0만 엔, 실세 GPI 2,167.2만 엔 [표면 6.57%]), ②접도 3.0m 노지상부지 조례 우회용 1F~3F 내계단 2개소 메조네트(계단로스 18%), ③LP가스 채택 및 전 12호 공실 리스업 리스크 존재. 2.90억~2.95억 엔(실세 표면 7.35%~7.47%) 네고 + 30년 융자 + 만실 인도/마스터리스 특약 조건부 매수(Conditional Buy)</t>
+          <t>C+ 등급 (61/100점 | 19.6/30점) — 오카다부동산(임대부·대주) 확정 모집도면 기준 만실 연수입 2,176.8만 엔(표면 6.60% / 관리비 제외 시 2,119.2만 엔·6.42%)으로 매매 마이소쿠(연 2,386.8만 엔·7.23%) 대비 연 -210.0만 엔(관리비 제외 시 -267.6만 엔) 하향 확정(2LDK 전 6호 호당 월 -2만 엔 인하, 106호 1DK 확정, AD100%+FR1개월 전용가). 호가 3.30억 엔 매수 보류 · 2.90억~2.95억 엔(모집가 기준 표면 7.38%~7.51%) 지가 네고 + 30년 융자 + 만실 인도/마스터리스 특약 조건부 매수(Conditional Buy)</t>
         </is>
       </c>
       <c r="CW15" s="0" t="inlineStr">
@@ -7721,12 +7721,12 @@
       </c>
       <c r="CX15" s="0" t="inlineStr">
         <is>
-          <t>조건부 매수 (61 / 100점 — 호가 3.30억 엔 보류 · 포털 실세 반영 2.90억~2.95억 엔 네고 및 30년 융자 필수)</t>
+          <t>조건부 매수 (61 / 100점 — 오카다부동산 확정 모집가[연 2,176.8만 엔·표면 6.60%, 임대료만 6.42%] 반영 2.90억~2.95억 엔 네고 및 30년 융자 필수)</t>
         </is>
       </c>
       <c r="CY15" s="0" t="inlineStr">
         <is>
-          <t>조건부 매수 (61 / 100점 — 호가 3.30억 엔 보류 · 포털 실세 반영 2.90억~2.95억 엔 네고 및 30년 융자 필수)</t>
+          <t>조건부 매수 (61 / 100점 — 오카다부동산 확정 모집가[연 2,176.8만 엔·표면 6.60%, 임대료만 6.42%] 반영 2.90억~2.95억 엔 네고 및 30년 융자 필수)</t>
         </is>
       </c>
     </row>
@@ -20637,12 +20637,12 @@
       </c>
       <c r="F149" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (선행모집·시공중)</t>
         </is>
       </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (9월 하순~ 계약개시)</t>
         </is>
       </c>
       <c r="H149" s="0" t="inlineStr">
@@ -20666,17 +20666,17 @@
         <v>124000</v>
       </c>
       <c r="N149" s="0">
-        <v>122000</v>
+        <v>124000</v>
       </c>
       <c r="O149" s="0">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="P149" s="0">
         <v>45</v>
       </c>
       <c r="Q149" s="0" t="inlineStr">
         <is>
-          <t>1층 남서 모서리 (포털 12.0만+4천엔 모집 중)</t>
+          <t>오카다부동산 모집도면 확정 (12.0만+관리비 4천엔 / 예금1·멘테상각1·AD100%+FR1M)</t>
         </is>
       </c>
     </row>
@@ -20704,12 +20704,12 @@
       </c>
       <c r="F150" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (선행모집·시공중)</t>
         </is>
       </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (9월 하순~ 계약개시)</t>
         </is>
       </c>
       <c r="H150" s="0" t="inlineStr">
@@ -20733,17 +20733,17 @@
         <v>122000</v>
       </c>
       <c r="N150" s="0">
-        <v>119000</v>
+        <v>122000</v>
       </c>
       <c r="O150" s="0">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="P150" s="0">
         <v>45</v>
       </c>
       <c r="Q150" s="0" t="inlineStr">
         <is>
-          <t>1층 중간호실 (포털 11.8만+4천엔 모집 중)</t>
+          <t>오카다부동산 모집도면 확정 (11.8만+관리비 4천엔 / 예금1·멘테상각1·AD100%+FR1M)</t>
         </is>
       </c>
     </row>
@@ -20771,12 +20771,12 @@
       </c>
       <c r="F151" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (선행모집·시공중)</t>
         </is>
       </c>
       <c r="G151" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (9월 하순~ 계약개시)</t>
         </is>
       </c>
       <c r="H151" s="0" t="inlineStr">
@@ -20800,17 +20800,17 @@
         <v>122000</v>
       </c>
       <c r="N151" s="0">
-        <v>119000</v>
+        <v>122000</v>
       </c>
       <c r="O151" s="0">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="P151" s="0">
         <v>45</v>
       </c>
       <c r="Q151" s="0" t="inlineStr">
         <is>
-          <t>1층 중간호실 (포털 11.8만+4천엔 모집 중)</t>
+          <t>오카다부동산 모집도면 확정 (11.8만+관리비 4천엔 / 예금1·멘테상각1·AD100%+FR1M)</t>
         </is>
       </c>
     </row>
@@ -20838,12 +20838,12 @@
       </c>
       <c r="F152" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (선행모집·시공중)</t>
         </is>
       </c>
       <c r="G152" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (9월 하순~ 계약개시)</t>
         </is>
       </c>
       <c r="H152" s="0" t="inlineStr">
@@ -20867,17 +20867,17 @@
         <v>122000</v>
       </c>
       <c r="N152" s="0">
-        <v>119000</v>
+        <v>122000</v>
       </c>
       <c r="O152" s="0">
-        <v>-3000</v>
+        <v>0</v>
       </c>
       <c r="P152" s="0">
         <v>45</v>
       </c>
       <c r="Q152" s="0" t="inlineStr">
         <is>
-          <t>1층 중간호실 (포털 11.8만+4천엔 모집 중)</t>
+          <t>오카다부동산 모집도면 확정 (11.8만+관리비 4천엔 / 예금1·멘테상각1·AD100%+FR1M)</t>
         </is>
       </c>
     </row>
@@ -20905,12 +20905,12 @@
       </c>
       <c r="F153" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (선행모집·시공중)</t>
         </is>
       </c>
       <c r="G153" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (9월 하순~ 계약개시)</t>
         </is>
       </c>
       <c r="H153" s="0" t="inlineStr">
@@ -20934,17 +20934,17 @@
         <v>119000</v>
       </c>
       <c r="N153" s="0">
-        <v>117000</v>
+        <v>119000</v>
       </c>
       <c r="O153" s="0">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="P153" s="0">
         <v>45</v>
       </c>
       <c r="Q153" s="0" t="inlineStr">
         <is>
-          <t>1층 동측 중간 (포털 11.5만+4천엔 모집 중)</t>
+          <t>오카다부동산 모집도면 확정 (11.5만+관리비 4천엔 / 예금1·멘테상각1·AD100%+FR1M)</t>
         </is>
       </c>
     </row>
@@ -20972,12 +20972,12 @@
       </c>
       <c r="F154" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (선행모집·시공중)</t>
         </is>
       </c>
       <c r="G154" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (9월 하순~ 계약개시)</t>
         </is>
       </c>
       <c r="H154" s="0" t="inlineStr">
@@ -21001,17 +21001,17 @@
         <v>120000</v>
       </c>
       <c r="N154" s="0">
-        <v>118000</v>
+        <v>120000</v>
       </c>
       <c r="O154" s="0">
-        <v>-2000</v>
+        <v>0</v>
       </c>
       <c r="P154" s="0">
         <v>45</v>
       </c>
       <c r="Q154" s="0" t="inlineStr">
         <is>
-          <t>1층 북동 모서리 (포털 11.6만+4천엔 모집 중)</t>
+          <t>⚠️ 매매마이소쿠 1LDK 표기이나 오카다 모집도면상 1DK(DK7첩+양5첩) 확정 (11.6만+4천엔)</t>
         </is>
       </c>
     </row>
@@ -21039,12 +21039,12 @@
       </c>
       <c r="F155" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (완성전·선행모집)</t>
         </is>
       </c>
       <c r="G155" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (10월 상순~ 개시)</t>
         </is>
       </c>
       <c r="H155" s="0" t="inlineStr">
@@ -21056,7 +21056,7 @@
         <v>0.0</v>
       </c>
       <c r="J155" s="0">
-        <v>200000</v>
+        <v>180000</v>
       </c>
       <c r="K155" s="0">
         <v>4000</v>
@@ -21065,7 +21065,7 @@
         <v>0</v>
       </c>
       <c r="M155" s="0">
-        <v>204000</v>
+        <v>184000</v>
       </c>
       <c r="N155" s="0">
         <v>184000</v>
@@ -21078,7 +21078,7 @@
       </c>
       <c r="Q155" s="0" t="inlineStr">
         <is>
-          <t>⚠️ 포털 실모집가 17.5만~18.0만+4천엔으로 인하 (계단로스 반영)</t>
+          <t>⚠️ 매매마이소쿠(20.0만) 대비 -2.0만엔 인하 확정 (18.0만+4천엔 / 임대도면 면적 미기재)</t>
         </is>
       </c>
     </row>
@@ -21106,12 +21106,12 @@
       </c>
       <c r="F156" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (완성전·선행모집)</t>
         </is>
       </c>
       <c r="G156" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (10월 상순~ 개시)</t>
         </is>
       </c>
       <c r="H156" s="0" t="inlineStr">
@@ -21123,7 +21123,7 @@
         <v>0.0</v>
       </c>
       <c r="J156" s="0">
-        <v>195000</v>
+        <v>175000</v>
       </c>
       <c r="K156" s="0">
         <v>4000</v>
@@ -21132,20 +21132,20 @@
         <v>0</v>
       </c>
       <c r="M156" s="0">
-        <v>199000</v>
+        <v>179000</v>
       </c>
       <c r="N156" s="0">
-        <v>181000</v>
+        <v>179000</v>
       </c>
       <c r="O156" s="0">
-        <v>-18000</v>
+        <v>-20000</v>
       </c>
       <c r="P156" s="0">
         <v>75</v>
       </c>
       <c r="Q156" s="0" t="inlineStr">
         <is>
-          <t>⚠️ 포털 실모집가 17.5만+4천엔으로 인하 (부금0·예금0)</t>
+          <t>⚠️ 매매마이소쿠(19.5만) 대비 -2.0만엔 인하 확정 (17.5만+4천엔 / 임대도면 면적 미기재)</t>
         </is>
       </c>
     </row>
@@ -21173,12 +21173,12 @@
       </c>
       <c r="F157" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (완성전·선행모집)</t>
         </is>
       </c>
       <c r="G157" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (10월 상순~ 개시)</t>
         </is>
       </c>
       <c r="H157" s="0" t="inlineStr">
@@ -21190,7 +21190,7 @@
         <v>0.0</v>
       </c>
       <c r="J157" s="0">
-        <v>195000</v>
+        <v>175000</v>
       </c>
       <c r="K157" s="0">
         <v>4000</v>
@@ -21199,20 +21199,20 @@
         <v>0</v>
       </c>
       <c r="M157" s="0">
-        <v>199000</v>
+        <v>179000</v>
       </c>
       <c r="N157" s="0">
-        <v>181000</v>
+        <v>179000</v>
       </c>
       <c r="O157" s="0">
-        <v>-18000</v>
+        <v>-20000</v>
       </c>
       <c r="P157" s="0">
         <v>75</v>
       </c>
       <c r="Q157" s="0" t="inlineStr">
         <is>
-          <t>⚠️ 포털 실모집가 17.5만+4천엔으로 인하 (부금0·예금0)</t>
+          <t>⚠️ 매매마이소쿠(19.5만) 대비 -2.0만엔 인하 확정 (17.5만+4천엔 / 임대도면 면적 미기재)</t>
         </is>
       </c>
     </row>
@@ -21240,12 +21240,12 @@
       </c>
       <c r="F158" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (완성전·선행모집)</t>
         </is>
       </c>
       <c r="G158" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (10월 상순~ 개시)</t>
         </is>
       </c>
       <c r="H158" s="0" t="inlineStr">
@@ -21257,7 +21257,7 @@
         <v>0.0</v>
       </c>
       <c r="J158" s="0">
-        <v>195000</v>
+        <v>175000</v>
       </c>
       <c r="K158" s="0">
         <v>4000</v>
@@ -21266,20 +21266,20 @@
         <v>0</v>
       </c>
       <c r="M158" s="0">
-        <v>199000</v>
+        <v>179000</v>
       </c>
       <c r="N158" s="0">
-        <v>181000</v>
+        <v>179000</v>
       </c>
       <c r="O158" s="0">
-        <v>-18000</v>
+        <v>-20000</v>
       </c>
       <c r="P158" s="0">
         <v>75</v>
       </c>
       <c r="Q158" s="0" t="inlineStr">
         <is>
-          <t>⚠️ 포털 실모집가 17.5만+4천엔으로 인하 (부금0·예금0)</t>
+          <t>⚠️ 매매마이소쿠(19.5만) 대비 -2.0만엔 인하 확정 (17.5만+4천엔 / 임대도면 면적 미기재)</t>
         </is>
       </c>
     </row>
@@ -21307,12 +21307,12 @@
       </c>
       <c r="F159" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (완성전·선행모집)</t>
         </is>
       </c>
       <c r="G159" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (10월 상순~ 개시)</t>
         </is>
       </c>
       <c r="H159" s="0" t="inlineStr">
@@ -21324,7 +21324,7 @@
         <v>0.0</v>
       </c>
       <c r="J159" s="0">
-        <v>196000</v>
+        <v>176000</v>
       </c>
       <c r="K159" s="0">
         <v>4000</v>
@@ -21333,20 +21333,20 @@
         <v>0</v>
       </c>
       <c r="M159" s="0">
-        <v>200000</v>
+        <v>180000</v>
       </c>
       <c r="N159" s="0">
-        <v>182000</v>
+        <v>180000</v>
       </c>
       <c r="O159" s="0">
-        <v>-18000</v>
+        <v>-20000</v>
       </c>
       <c r="P159" s="0">
         <v>75</v>
       </c>
       <c r="Q159" s="0" t="inlineStr">
         <is>
-          <t>⚠️ 포털 실모집가 18.0만+4천엔으로 인하 (약 18.1첩 LDK)</t>
+          <t>⚠️ 매매마이소쿠(19.6만) 대비 -2.0만엔 인하 확정 (17.6만+4천엔 / 3층 18.1첩 LDK 배치)</t>
         </is>
       </c>
     </row>
@@ -21374,12 +21374,12 @@
       </c>
       <c r="F160" s="0" t="inlineStr">
         <is>
-          <t>공실 (신축모집중)</t>
+          <t>공실 (완성전·선행모집)</t>
         </is>
       </c>
       <c r="G160" s="0" t="inlineStr">
         <is>
-          <t>미입주 (신축 리스업 중)</t>
+          <t>미입주 (10월 상순~ 개시)</t>
         </is>
       </c>
       <c r="H160" s="0" t="inlineStr">
@@ -21391,7 +21391,7 @@
         <v>0.0</v>
       </c>
       <c r="J160" s="0">
-        <v>200000</v>
+        <v>180000</v>
       </c>
       <c r="K160" s="0">
         <v>4000</v>
@@ -21400,20 +21400,20 @@
         <v>0</v>
       </c>
       <c r="M160" s="0">
-        <v>204000</v>
+        <v>184000</v>
       </c>
       <c r="N160" s="0">
-        <v>183000</v>
+        <v>184000</v>
       </c>
       <c r="O160" s="0">
-        <v>-21000</v>
+        <v>-20000</v>
       </c>
       <c r="P160" s="0">
         <v>75</v>
       </c>
       <c r="Q160" s="0" t="inlineStr">
         <is>
-          <t>⚠️ 포털 실모집가 18.0만~19.5만+4천엔으로 인하 (북동 모서리)</t>
+          <t>⚠️ 매매마이소쿠(20.0만) 대비 -2.0만엔 인하 확정 (18.0만+4천엔 / 3층 욕실·세면실 배치)</t>
         </is>
       </c>
     </row>
@@ -47967,7 +47967,7 @@
       </c>
       <c r="H466" s="0" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>COLLECTED</t>
         </is>
       </c>
       <c r="I466" s="0" t="inlineStr">
@@ -48158,116 +48158,116 @@
       </c>
     </row>
     <row r="470">
-      <c r="A470" s="3" t="inlineStr">
+      <c r="A470" s="0" t="inlineStr">
         <is>
           <t>karen-residence-nishitakenotsuka</t>
         </is>
       </c>
-      <c r="B470" s="3" t="inlineStr">
+      <c r="B470" s="0" t="inlineStr">
         <is>
           <t>CHK_14</t>
         </is>
       </c>
-      <c r="C470" s="3" t="inlineStr">
+      <c r="C470" s="0" t="inlineStr">
         <is>
           <t>3.건물/적법</t>
         </is>
       </c>
-      <c r="D470" s="3" t="inlineStr">
+      <c r="D470" s="0" t="inlineStr">
         <is>
           <t>has_confirm_cert</t>
         </is>
       </c>
-      <c r="E470" s="3" t="inlineStr">
+      <c r="E470" s="0" t="inlineStr">
         <is>
           <t>건축확인필증(確認済証) 및 대장 유무</t>
         </is>
       </c>
-      <c r="F470" s="3" t="inlineStr">
+      <c r="F470" s="0" t="inlineStr">
         <is>
           <t>建築確認済証・台帳記載事項証明</t>
         </is>
       </c>
-      <c r="G470" s="3" t="inlineStr">
+      <c r="G470" s="0" t="inlineStr">
         <is>
           <t>보유 확실 (2026년 신축 — 단, 용도가 『나가야』인지 『공동주택』인지 사본 확인 필수)</t>
         </is>
       </c>
-      <c r="H470" s="3" t="inlineStr">
-        <is>
-          <t>ESTIMATED</t>
-        </is>
-      </c>
-      <c r="I470" s="3" t="inlineStr">
-        <is>
-          <t>표준산식 역산 추정</t>
-        </is>
-      </c>
-      <c r="J470" s="3" t="inlineStr">
-        <is>
-          <t>건축확인필증 또는 대장기재사항증명서 사본 요청</t>
-        </is>
-      </c>
-      <c r="K470" s="3" t="inlineStr">
-        <is>
-          <t>建築確認済証または台帳記載事項証明書の写しのご共有</t>
+      <c r="H470" s="0" t="inlineStr">
+        <is>
+          <t>COLLECTED</t>
+        </is>
+      </c>
+      <c r="I470" s="0" t="inlineStr">
+        <is>
+          <t>건축확인대장</t>
+        </is>
+      </c>
+      <c r="J470" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K470" s="0" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
     <row r="471">
-      <c r="A471" s="3" t="inlineStr">
+      <c r="A471" s="0" t="inlineStr">
         <is>
           <t>karen-residence-nishitakenotsuka</t>
         </is>
       </c>
-      <c r="B471" s="3" t="inlineStr">
+      <c r="B471" s="0" t="inlineStr">
         <is>
           <t>CHK_15</t>
         </is>
       </c>
-      <c r="C471" s="3" t="inlineStr">
+      <c r="C471" s="0" t="inlineStr">
         <is>
           <t>3.건물/적법</t>
         </is>
       </c>
-      <c r="D471" s="3" t="inlineStr">
+      <c r="D471" s="0" t="inlineStr">
         <is>
           <t>has_inspection_cert</t>
         </is>
       </c>
-      <c r="E471" s="3" t="inlineStr">
+      <c r="E471" s="0" t="inlineStr">
         <is>
           <t>준공검사필증(検査済証) 취득 여부</t>
         </is>
       </c>
-      <c r="F471" s="3" t="inlineStr">
+      <c r="F471" s="0" t="inlineStr">
         <is>
           <t>検査済証の有無</t>
         </is>
       </c>
-      <c r="G471" s="3" t="inlineStr">
+      <c r="G471" s="0" t="inlineStr">
         <is>
           <t>보유 확실 (2026년 신축 — 준공검사필증 및 열화등급 3급 상당 증명서 원본 징구 필수)</t>
         </is>
       </c>
-      <c r="H471" s="3" t="inlineStr">
-        <is>
-          <t>ESTIMATED</t>
-        </is>
-      </c>
-      <c r="I471" s="3" t="inlineStr">
-        <is>
-          <t>표준산식 역산 추정</t>
-        </is>
-      </c>
-      <c r="J471" s="3" t="inlineStr">
-        <is>
-          <t>준공검사필증(検査済証) 교부 유무 및 번호 확인 (은행융자 필수)</t>
-        </is>
-      </c>
-      <c r="K471" s="3" t="inlineStr">
-        <is>
-          <t>検査済証の有無および交付番号のご確認（融資審査上必須）</t>
+      <c r="H471" s="0" t="inlineStr">
+        <is>
+          <t>COLLECTED</t>
+        </is>
+      </c>
+      <c r="I471" s="0" t="inlineStr">
+        <is>
+          <t>검사필증/대장</t>
+        </is>
+      </c>
+      <c r="J471" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K471" s="0" t="inlineStr">
+        <is>
+          <t/>
         </is>
       </c>
     </row>
@@ -48361,12 +48361,12 @@
       </c>
       <c r="G473" s="0" t="inlineStr">
         <is>
-          <t>23868000</t>
+          <t>21768000</t>
         </is>
       </c>
       <c r="H473" s="0" t="inlineStr">
         <is>
-          <t>COLLECTED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="I473" s="0" t="inlineStr">
@@ -48418,7 +48418,7 @@
       </c>
       <c r="G474" s="0" t="inlineStr">
         <is>
-          <t>1LDK(32.57~33.01㎡)×6호 [1층] + 2LDK 메조네트(70.48~71.76㎡, 1F현관+2·3F)×6호</t>
+          <t>1LDK(32.78~33.01㎡)×5호 + 1DK(32.57㎡)×1호 [1층] + 2LDK 메조네트(70.48~71.76㎡, 임대도면 면적 미기재)×6호 [2~3층]</t>
         </is>
       </c>
       <c r="H474" s="0" t="inlineStr">
@@ -48443,59 +48443,59 @@
       </c>
     </row>
     <row r="475">
-      <c r="A475" s="0" t="inlineStr">
+      <c r="A475" s="2" t="inlineStr">
         <is>
           <t>karen-residence-nishitakenotsuka</t>
         </is>
       </c>
-      <c r="B475" s="0" t="inlineStr">
+      <c r="B475" s="2" t="inlineStr">
         <is>
           <t>CHK_19</t>
         </is>
       </c>
-      <c r="C475" s="0" t="inlineStr">
+      <c r="C475" s="2" t="inlineStr">
         <is>
           <t>4.렌트롤</t>
         </is>
       </c>
-      <c r="D475" s="0" t="inlineStr">
+      <c r="D475" s="2" t="inlineStr">
         <is>
           <t>rent_roll_contract_dates</t>
         </is>
       </c>
-      <c r="E475" s="0" t="inlineStr">
+      <c r="E475" s="2" t="inlineStr">
         <is>
           <t>호실별 계약시작일(契約始期) 및 갱신주기</t>
         </is>
       </c>
-      <c r="F475" s="0" t="inlineStr">
+      <c r="F475" s="2" t="inlineStr">
         <is>
           <t>各戸の契約始期・更新時期</t>
         </is>
       </c>
-      <c r="G475" s="0" t="inlineStr">
+      <c r="G475" s="2" t="inlineStr">
         <is>
           <t>[미수집 - 계약시작일 미기재]</t>
         </is>
       </c>
-      <c r="H475" s="0" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-      <c r="I475" s="0" t="inlineStr">
-        <is>
-          <t>렌트롤 상세판</t>
-        </is>
-      </c>
-      <c r="J475" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K475" s="0" t="inlineStr">
-        <is>
-          <t/>
+      <c r="H475" s="2" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="I475" s="2" t="inlineStr">
+        <is>
+          <t>미수령 (중개사 요청 필요)</t>
+        </is>
+      </c>
+      <c r="J475" s="2" t="inlineStr">
+        <is>
+          <t>렌트롤상 호실별 최초 계약시작일(입주일) 기재본 요청</t>
+        </is>
+      </c>
+      <c r="K475" s="2" t="inlineStr">
+        <is>
+          <t>レントロールにおける各戸の契約始期（入居年月）のご教示</t>
         </is>
       </c>
     </row>
@@ -48537,7 +48537,7 @@
       </c>
       <c r="H476" s="0" t="inlineStr">
         <is>
-          <t>VERIFIED</t>
+          <t>COLLECTED</t>
         </is>
       </c>
       <c r="I476" s="0" t="inlineStr">
@@ -59386,16 +59386,16 @@
       </c>
       <c r="E132" s="0" t="inlineStr">
         <is>
-          <t>**니시타케노츠카 2초메 카렌 레지던스(西竹の塚2丁目 カレンレジデンス)**는 도부 스카이트리 라인 『타케노츠카』역 도보 3분 근린상업지역 토지 384.62㎡(116.35평) 위에 신축된 **목조 3층 건 12세대(1LDK×6호 + 2LDK 메조네트×6호, 연면적 605.17㎡)** 대형 아파트를 대상으로 합니다.
-- **3단계 렌트롤 감사 적발**: 마이소쿠 헤드라인(연 2,386.8만 엔 / 7.23%)과 표 합산(연 2,320.8만 엔 / 7.03%) 간 연 -66만 엔 산술 오차가 존재하며, 2026년 10월 현재 SUUMO 등 실제 임대 포털에서는 2LDK가 이미 **월 17.5만~18.0만 엔(부금0·예금0)**으로 인하 모집 중이어서 **실전 성약 기준 만실 연수입(GPI)은 2,167.2만 엔(표면 6.57%, 실효 NOI 1,692.5만 엔 [Cap 5.13%])**으로 하락합니다.
-- **최종 판정**: **조건부 매수(Conditional Buy, 61/100점 | 19.6/30점, C+ 등급)** — 호가 3.30억 엔 매수는 보류하며, **2억 9,000만~2억 9,500만 엔(실세 표면 7.35%~7.47%) 지가 네고 + 30년 융자 특약 + 만실 인도(또는 1년 마스터리스) 특약** 성사 시에만 매수를 권고합니다.</t>
+          <t>**니시타케노츠카 2초메 카렌 레지던스(西竹の塚2丁目 カレンレジデンス)**는 도부 스카이트리 라인 『타케노츠카』역 도보 3분 근린상업지역 토지 384.62㎡(116.35평) 위에 신축된 **목조 3층 건 12세대(1층: 1LDK×5호+1DK×1호[197.39㎡], 2~3층: 2LDK 메조네트×6호, 연면적 605.17㎡)** 대형 아파트를 대상으로 합니다.
+- **오카다부동산(임대부·대주) 모집도면 7매 및 확정 렌트롤 대조 적발**: 매매 마이소쿠 헤드라인(연 2,386.8만 엔 / 7.23%) 및 표 합산(연 2,320.8만 엔 / 7.03%)과 달리, 실제 임대 모집도면에서는 **2~3층 2LDK 6세대 전 호실이 일괄 월 -20,000엔 인하(17.5만~18.0만 엔+관리비 4,000엔)**되어 **확정 만실 연수입(GPI)은 관리비 포함 2,176.8만 엔(표면 6.60%, 연 -210.0만 엔 감소 / 실효 NOI 1,701.1만 엔 [Cap 5.15%]), 임대료만 합산 시 2,119.2만 엔(표면 6.42%, 연 -267.6만 엔 감소)**으로 확정되었습니다.
+- **최종 판정**: **조건부 매수(Conditional Buy, 61/100점 | 19.6/30점, C+ 등급)** — 호가 3.30억 엔 매수는 보류하며, **2억 9,000만~2억 9,500만 엔(모집확정 기준 표면 7.38%~7.51%) 지가 네고 + 30년 융자 특약 + 만실 인도(AD100%+FR1개월 매도자 부담) 특약** 성사 시에만 매수를 권고합니다.</t>
         </is>
       </c>
       <c r="F132" s="0" t="inlineStr">
         <is>
-          <t>**西竹の塚2丁目 カレンレジデンス**は、東武スカイツリーライン『竹ノ塚』駅徒歩3分の近隣商業地域（土地384.62㎡・116.35坪）に新築された**木造3階建・全12戸（1LDK×6戸＋2LDKメゾネット×6戸、延床605.17㎡）**の一棟アパートです。
-- **3段階レントロール監査**: マイソク表面記載（年2,386.8万円 / 7.23%）と賃料表実合算（年2,320.8万円 / 7.03%）に年▲66万円の算術不一致がある上、現行SUUMO等の賃貸ポータルでは2LDKが既に**月17.5万〜18.0万円（敷0・礼0）**へ値下げ募集されており、**実勢満室GPIは年2,167.2万円（表面6.57%・実効NOI 1,692.5万円［Cap 5.13%］）**となります。
-- **最終判定**: **条件付推奨（Conditional Buy、61/100点｜19.6/30点、ランクC+）** — 売出3.30億円での買付は見送り、**2億9,000万〜2億9,500万円（実勢表面7.35%〜7.47%）への指値交渉＋30年融資特約＋満室引渡（または家賃保証）特約**を必須条件とします。</t>
+          <t>**西竹の塚2丁目 カレンレジデンス**は、東武スカイツリーライン『竹ノ塚』駅徒歩3分の近隣商業地域（土地384.62㎡・116.35坪）に新築された**木造3階建・全12戸（1階：1LDK×5戸＋1DK×1戸［計197.39㎡］、2〜3階：2LDKメゾネット×6戸、延床605.17㎡）**の一棟アパートです。
+- **岡田不動産（賃貸部・貸主）募集図面（全7枚）および確定レントロール監査**: 売買マイソク表面記載（年2,386.8万円 / 7.23%）および表合算（年2,320.8万円 / 7.03%）に対し、実際の賃貸募集図面では**2〜3階2LDK全6戸が一律月▲20,000円引き下げ（17.5万〜18.0万円＋管理費4,000円）**て募集されており、**確定満室GPIは管理費込みで年2,176.8万円（表面6.60%・年▲210.0万円減 ／ 実効NOI 1,701.1万円［Cap 5.15%］）、賃料のみでは年2,119.2万円（表面6.42%・年▲267.6万円減）**となることが確定しました。
+- **最終判定**: **条件付推奨（Conditional Buy、61/100点｜19.6/30点、ランクC+）** — 売出3.30億円での買付は見送り、**2億9,000万〜2億9,500万円（募集図面確定ベース表面7.38%〜7.51%）への指値交渉＋30年融資特約＋満室引渡（初期AD100%＋FR1ヶ月売主負担）特約**を必須条件とします。</t>
         </is>
       </c>
     </row>
@@ -59522,14 +59522,16 @@
       </c>
       <c r="E136" s="0" t="inlineStr">
         <is>
-          <t>- **왜 2LDK(70.48㎡)가 포털에서 월 17.5만~18.0만 엔으로 할인 모집 중인가?**: 도쿄도 건축안전조례(접도 3.0m 제한)를 충족하기 위해 201~206호를 『1층 전용현관 → 내계단 → 2층 LDK → 내계단 → 3층 침실 2개』의 **3개층 수직 겹침나가야(트리플렛 메조네트)**로 설계하여, 70.48㎡ 중 약 12~15㎡(18~20%)가 2개의 계단실로 소모됩니다.
-- **3단계 수입 비교**: ①마이소쿠 헤드라인 **연 2,386.8만 엔(7.23%)** vs ②마이소쿠 표 실제 합산 **연 2,320.8만 엔(7.03%, -66만 엔 오차)** vs ③실전 포털(SUUMO) 모집 실세 반영 **연 2,167.2만 엔(6.57%, -219.6만 엔 감소)**.</t>
+          <t>- **오카다부동산(임대부) 모집도면 7매 정밀 대조**: 1층 `106호`가 매매 마이소쿠(1LDK)와 달리 **1DK(DK 약7첩+양실 약5첩)**로 확정되었고, 2~3층 메조네트(`201~206호`)는 계단실 로스(약 12~15㎡)로 인해 임대 모집도면에 **전유면적 『미기재(記載なし)』**로 등록되어 있으며 평면은 ①`201~204호`(2F LDK 12.2첩 / 3F 양실 2개+WIC 2개), ②`205호`(2F 양실 2개+욕실 / **3F 대형 LDK 18.1첩**), ③`206호`(2F LDK 14.1첩 / 3F 양실 2개+욕실)의 3타입으로 구성됩니다.
+- **4단계 수입 비교**: ①매매 마이소쿠 헤드라인 **연 2,386.8만 엔(7.23%)** vs ②매매 마이소쿠 표 합산 **연 2,320.8만 엔(7.03%)** vs ③**오카다부동산 모집도면 확정(관리비 포함) 연 2,176.8만 엔(6.60%, 월 181.4만 엔)** vs ④**모집도면 확정(임대료만) 연 2,119.2만 엔(6.42%, 월 176.6만 엔)**.
+- **초기 모집 조건**: 예금 1개월 + 멘테넌스 비용 1개월(퇴거 시 전액 상각) + 조기해약 위약금(1년 미만 1개월, 2년 미만 0.5개월) 및 객부 중개사 인센티브 **`AD 100% + FR 1개월(전용 가능)`** 설정.</t>
         </is>
       </c>
       <c r="F136" s="0" t="inlineStr">
         <is>
-          <t>- **なぜ2LDK（70.48㎡）がポータルで月17.5万〜18.0万円へ値下げ募集されているのか？**: 東京都建築安全条例（接道3.0m制限）をクリアするため、201〜206号室を『1階専用玄関→内階段→2階LDK→内階段→3階洋室2室』の**3層トリプレット型メゾネット（重ね長屋）**として設計しており、70.48㎡のうち約12〜15㎡（18〜20%）が2つの内階段に消費されています。
-- **3段階収入比較**: ①マイソク表面記載 **年2,386.8万円（7.23%）** vs ②マイソク表実合算 **年2,320.8万円（7.03%、▲66万円誤差）** vs ③現行ポータル（SUUMO）実勢反映 **年2,167.2万円（6.57%、▲219.6万円減）**。</t>
+          <t>- **岡田不動産（賃貸部）募集図面（全7枚）の精密照合**: 1階`106号室`が売買マイソク（1LDK）と異なり**1DK（DK約7帖＋洋室約5帖）**で確定。2〜3階メゾネット（`201〜206号室`）は階段ロス（約12〜15㎡）を考慮して賃貸募集図面では**専有面積「記載なし」**となっており、間取りは①`201〜204号室`（2F LDK12.2帖／3F 洋室2室＋WIC2ヶ所）、②`205号室`（2F 洋室2室＋水回り／**3F 大型LDK18.1帖**）、③`206号室`（2F LDK14.1帖／3F 洋室2室＋水回り）の3タイプで構成されています。
+- **4段階収入比較**: ①売買マイソク表面 **年2,386.8万円（7.23%）** vs ②売買マイソク表合算 **年2,320.8万円（7.03%）** vs ③**岡田不動産 募集図面確定［管理費込］年2,176.8万円（6.60%・月181.4万円）** vs ④**募集図面確定［賃料のみ］年2,119.2万円（6.42%・月176.6万円）**。
+- **募集・契約条件**: 礼金1ヶ月＋メンテナンス費用1ヶ月（退去時全額償却）＋早期解約違約金（1年未満1ヶ月・2年未満0.5ヶ月）および客付インセンティブ**『AD100%＋FR1ヶ月（転用可）』**。</t>
         </is>
       </c>
     </row>

</xml_diff>